<commit_message>
Update refactor-safe ETF PE history
</commit_message>
<xml_diff>
--- a/etf_analyst_target_outputs/ETF_PE_history.xlsx
+++ b/etf_analyst_target_outputs/ETF_PE_history.xlsx
@@ -2835,10 +2835,10 @@
         <v>8</v>
       </c>
       <c r="C93">
-        <v>20.49046763366244</v>
+        <v>20.52198379076916</v>
       </c>
       <c r="D93">
-        <v>15.9545172814726</v>
+        <v>15.95436859937961</v>
       </c>
       <c r="E93">
         <v>0.9241000000000001</v>
@@ -2850,7 +2850,7 @@
         <v>0.5088591433601022</v>
       </c>
       <c r="H93">
-        <v>0.9412999999999999</v>
+        <v>0.9648999999999999</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -5409,10 +5409,10 @@
         <v>9</v>
       </c>
       <c r="C192">
-        <v>43.61473802848987</v>
+        <v>43.62323654820898</v>
       </c>
       <c r="D192">
-        <v>21.60105411248841</v>
+        <v>21.59885776580763</v>
       </c>
       <c r="E192">
         <v>0.9359</v>
@@ -5435,7 +5435,7 @@
         <v>10</v>
       </c>
       <c r="C193">
-        <v>6.439322817595627</v>
+        <v>6.439182551815224</v>
       </c>
       <c r="D193">
         <v>4.814996520798841</v>
@@ -8012,7 +8012,7 @@
         <v>28.36132882340183</v>
       </c>
       <c r="D292">
-        <v>23.82082574398114</v>
+        <v>23.81322164551797</v>
       </c>
       <c r="E292">
         <v>1.0002</v>
@@ -8035,10 +8035,10 @@
         <v>12</v>
       </c>
       <c r="C293">
-        <v>26.0155859506134</v>
+        <v>26.01446520788588</v>
       </c>
       <c r="D293">
-        <v>18.90897872248692</v>
+        <v>18.89745365058819</v>
       </c>
       <c r="E293">
         <v>0.9994999999999998</v>
@@ -8047,7 +8047,7 @@
         <v>0.9994999999999998</v>
       </c>
       <c r="G293">
-        <v>0.1270096895940624</v>
+        <v>0.1270095884355344</v>
       </c>
       <c r="H293">
         <v>0.9994999999999998</v>
@@ -10609,22 +10609,22 @@
         <v>13</v>
       </c>
       <c r="C392">
-        <v>31.43344621747044</v>
+        <v>31.48929813457532</v>
       </c>
       <c r="D392">
-        <v>20.3737089318342</v>
+        <v>20.35973635048795</v>
       </c>
       <c r="E392">
-        <v>0.9920256499999999</v>
+        <v>0.9923586000000001</v>
       </c>
       <c r="F392">
-        <v>0.9920256499999999</v>
+        <v>0.9923586000000001</v>
       </c>
       <c r="G392">
         <v>0.2053733085798772</v>
       </c>
       <c r="H392">
-        <v>0.9938315200000001</v>
+        <v>0.9922818</v>
       </c>
     </row>
     <row r="393" spans="1:8">
@@ -13183,10 +13183,10 @@
         <v>14</v>
       </c>
       <c r="C491">
-        <v>27.76463794596328</v>
+        <v>27.76661697585746</v>
       </c>
       <c r="D491">
-        <v>16.63635825605493</v>
+        <v>16.63467050331904</v>
       </c>
       <c r="E491">
         <v>0.9993</v>
@@ -15731,10 +15731,10 @@
         <v>15</v>
       </c>
       <c r="C589">
-        <v>33.11011225677496</v>
+        <v>33.11890811474259</v>
       </c>
       <c r="D589">
-        <v>18.01962019801299</v>
+        <v>18.01894893197226</v>
       </c>
       <c r="E589">
         <v>0.9987</v>
@@ -18305,10 +18305,10 @@
         <v>16</v>
       </c>
       <c r="C688">
-        <v>28.01997681258285</v>
+        <v>28.01843343721627</v>
       </c>
       <c r="D688">
-        <v>16.56578967998621</v>
+        <v>16.56422974318342</v>
       </c>
       <c r="E688">
         <v>1.00016299</v>
@@ -20879,7 +20879,7 @@
         <v>24.02189394374583</v>
       </c>
       <c r="D787">
-        <v>22.51376891213164</v>
+        <v>22.5071894225957</v>
       </c>
       <c r="E787">
         <v>1</v>
@@ -23450,22 +23450,22 @@
         <v>18</v>
       </c>
       <c r="C886">
-        <v>35.65030210761727</v>
+        <v>35.75278262761136</v>
       </c>
       <c r="D886">
-        <v>19.44323284999984</v>
+        <v>19.45761115315375</v>
       </c>
       <c r="E886">
-        <v>0.99927994</v>
+        <v>0.99727644</v>
       </c>
       <c r="F886">
-        <v>0.99927994</v>
+        <v>0.99727644</v>
       </c>
       <c r="G886">
         <v>0.3529568954465609</v>
       </c>
       <c r="H886">
-        <v>0.99570457</v>
+        <v>0.99927994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mirror refactor-safe ETF PE history to main
</commit_message>
<xml_diff>
--- a/etf_analyst_target_outputs/ETF_PE_history.xlsx
+++ b/etf_analyst_target_outputs/ETF_PE_history.xlsx
@@ -2835,10 +2835,10 @@
         <v>8</v>
       </c>
       <c r="C93">
-        <v>20.49046763366244</v>
+        <v>20.52198379076916</v>
       </c>
       <c r="D93">
-        <v>15.9545172814726</v>
+        <v>15.95436859937961</v>
       </c>
       <c r="E93">
         <v>0.9241000000000001</v>
@@ -2850,7 +2850,7 @@
         <v>0.5088591433601022</v>
       </c>
       <c r="H93">
-        <v>0.9412999999999999</v>
+        <v>0.9648999999999999</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -5409,10 +5409,10 @@
         <v>9</v>
       </c>
       <c r="C192">
-        <v>43.61473802848987</v>
+        <v>43.62323654820898</v>
       </c>
       <c r="D192">
-        <v>21.60105411248841</v>
+        <v>21.59885776580763</v>
       </c>
       <c r="E192">
         <v>0.9359</v>
@@ -5435,7 +5435,7 @@
         <v>10</v>
       </c>
       <c r="C193">
-        <v>6.439322817595627</v>
+        <v>6.439182551815224</v>
       </c>
       <c r="D193">
         <v>4.814996520798841</v>
@@ -8012,7 +8012,7 @@
         <v>28.36132882340183</v>
       </c>
       <c r="D292">
-        <v>23.82082574398114</v>
+        <v>23.81322164551797</v>
       </c>
       <c r="E292">
         <v>1.0002</v>
@@ -8035,10 +8035,10 @@
         <v>12</v>
       </c>
       <c r="C293">
-        <v>26.0155859506134</v>
+        <v>26.01446520788588</v>
       </c>
       <c r="D293">
-        <v>18.90897872248692</v>
+        <v>18.89745365058819</v>
       </c>
       <c r="E293">
         <v>0.9994999999999998</v>
@@ -8047,7 +8047,7 @@
         <v>0.9994999999999998</v>
       </c>
       <c r="G293">
-        <v>0.1270096895940624</v>
+        <v>0.1270095884355344</v>
       </c>
       <c r="H293">
         <v>0.9994999999999998</v>
@@ -10609,22 +10609,22 @@
         <v>13</v>
       </c>
       <c r="C392">
-        <v>31.43344621747044</v>
+        <v>31.48929813457532</v>
       </c>
       <c r="D392">
-        <v>20.3737089318342</v>
+        <v>20.35973635048795</v>
       </c>
       <c r="E392">
-        <v>0.9920256499999999</v>
+        <v>0.9923586000000001</v>
       </c>
       <c r="F392">
-        <v>0.9920256499999999</v>
+        <v>0.9923586000000001</v>
       </c>
       <c r="G392">
         <v>0.2053733085798772</v>
       </c>
       <c r="H392">
-        <v>0.9938315200000001</v>
+        <v>0.9922818</v>
       </c>
     </row>
     <row r="393" spans="1:8">
@@ -13183,10 +13183,10 @@
         <v>14</v>
       </c>
       <c r="C491">
-        <v>27.76463794596328</v>
+        <v>27.76661697585746</v>
       </c>
       <c r="D491">
-        <v>16.63635825605493</v>
+        <v>16.63467050331904</v>
       </c>
       <c r="E491">
         <v>0.9993</v>
@@ -15731,10 +15731,10 @@
         <v>15</v>
       </c>
       <c r="C589">
-        <v>33.11011225677496</v>
+        <v>33.11890811474259</v>
       </c>
       <c r="D589">
-        <v>18.01962019801299</v>
+        <v>18.01894893197226</v>
       </c>
       <c r="E589">
         <v>0.9987</v>
@@ -18305,10 +18305,10 @@
         <v>16</v>
       </c>
       <c r="C688">
-        <v>28.01997681258285</v>
+        <v>28.01843343721627</v>
       </c>
       <c r="D688">
-        <v>16.56578967998621</v>
+        <v>16.56422974318342</v>
       </c>
       <c r="E688">
         <v>1.00016299</v>
@@ -20879,7 +20879,7 @@
         <v>24.02189394374583</v>
       </c>
       <c r="D787">
-        <v>22.51376891213164</v>
+        <v>22.5071894225957</v>
       </c>
       <c r="E787">
         <v>1</v>
@@ -23450,22 +23450,22 @@
         <v>18</v>
       </c>
       <c r="C886">
-        <v>35.65030210761727</v>
+        <v>35.75278262761136</v>
       </c>
       <c r="D886">
-        <v>19.44323284999984</v>
+        <v>19.45761115315375</v>
       </c>
       <c r="E886">
-        <v>0.99927994</v>
+        <v>0.99727644</v>
       </c>
       <c r="F886">
-        <v>0.99927994</v>
+        <v>0.99727644</v>
       </c>
       <c r="G886">
         <v>0.3529568954465609</v>
       </c>
       <c r="H886">
-        <v>0.99570457</v>
+        <v>0.99927994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ETF PE history
</commit_message>
<xml_diff>
--- a/etf_analyst_target_outputs/ETF_PE_history.xlsx
+++ b/etf_analyst_target_outputs/ETF_PE_history.xlsx
@@ -2835,22 +2835,22 @@
         <v>8</v>
       </c>
       <c r="C93">
-        <v>20.52198379076916</v>
+        <v>20.34793925835714</v>
       </c>
       <c r="D93">
-        <v>15.95436859937961</v>
+        <v>15.9972197451635</v>
       </c>
       <c r="E93">
-        <v>0.9241000000000001</v>
+        <v>0.9238999999999999</v>
       </c>
       <c r="F93">
-        <v>0.9055000000000001</v>
+        <v>0.9056999999999999</v>
       </c>
       <c r="G93">
-        <v>0.5088591433601022</v>
+        <v>0.5770014382754669</v>
       </c>
       <c r="H93">
-        <v>0.9648999999999999</v>
+        <v>0.9841000000000001</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -5409,7 +5409,7 @@
         <v>9</v>
       </c>
       <c r="C192">
-        <v>43.62323654820898</v>
+        <v>43.69502672698427</v>
       </c>
       <c r="D192">
         <v>21.59885776580763</v>
@@ -5421,7 +5421,7 @@
         <v>0.9359</v>
       </c>
       <c r="G192">
-        <v>0.5486388138414446</v>
+        <v>0.6077407522088676</v>
       </c>
       <c r="H192">
         <v>0.9359</v>
@@ -5435,22 +5435,19 @@
         <v>10</v>
       </c>
       <c r="C193">
-        <v>6.439182551815224</v>
+        <v>6.45778759942359</v>
       </c>
       <c r="D193">
-        <v>4.814996520798841</v>
+        <v>4.845117594846442</v>
       </c>
       <c r="E193">
-        <v>0.9393999999999999</v>
+        <v>0.9406</v>
       </c>
       <c r="F193">
-        <v>0.9065999999999999</v>
-      </c>
-      <c r="G193">
-        <v>1.150576378627939</v>
+        <v>0.9083</v>
       </c>
       <c r="H193">
-        <v>0.9393999999999999</v>
+        <v>0.9406</v>
       </c>
     </row>
     <row r="194" spans="1:8">
@@ -8009,10 +8006,10 @@
         <v>11</v>
       </c>
       <c r="C292">
-        <v>28.36132882340183</v>
+        <v>28.2749625131891</v>
       </c>
       <c r="D292">
-        <v>23.81322164551797</v>
+        <v>23.71546940427201</v>
       </c>
       <c r="E292">
         <v>1.0002</v>
@@ -8021,7 +8018,7 @@
         <v>1.0002</v>
       </c>
       <c r="G292">
-        <v>0.0944146643153887</v>
+        <v>0.1012735051227174</v>
       </c>
       <c r="H292">
         <v>1.0002</v>
@@ -8035,22 +8032,22 @@
         <v>12</v>
       </c>
       <c r="C293">
-        <v>26.01446520788588</v>
+        <v>26.00344681339427</v>
       </c>
       <c r="D293">
-        <v>18.89745365058819</v>
+        <v>18.89200667321541</v>
       </c>
       <c r="E293">
-        <v>0.9994999999999998</v>
+        <v>0.9994999999999999</v>
       </c>
       <c r="F293">
-        <v>0.9994999999999998</v>
+        <v>0.9994999999999999</v>
       </c>
       <c r="G293">
-        <v>0.1270095884355344</v>
+        <v>0.1336549465707042</v>
       </c>
       <c r="H293">
-        <v>0.9994999999999998</v>
+        <v>0.9994999999999999</v>
       </c>
     </row>
     <row r="294" spans="1:8">
@@ -10609,22 +10606,22 @@
         <v>13</v>
       </c>
       <c r="C392">
-        <v>31.48929813457532</v>
+        <v>32.12042490092579</v>
       </c>
       <c r="D392">
-        <v>20.35973635048795</v>
+        <v>20.60550384270372</v>
       </c>
       <c r="E392">
-        <v>0.9923586000000001</v>
+        <v>0.9899363099999999</v>
       </c>
       <c r="F392">
-        <v>0.9923586000000001</v>
+        <v>0.9899363099999999</v>
       </c>
       <c r="G392">
-        <v>0.2053733085798772</v>
+        <v>0.2160563582197161</v>
       </c>
       <c r="H392">
-        <v>0.9922818</v>
+        <v>0.99785168</v>
       </c>
     </row>
     <row r="393" spans="1:8">
@@ -13183,10 +13180,10 @@
         <v>14</v>
       </c>
       <c r="C491">
-        <v>27.76661697585746</v>
+        <v>35.82097771612316</v>
       </c>
       <c r="D491">
-        <v>16.63467050331904</v>
+        <v>17.74198654168397</v>
       </c>
       <c r="E491">
         <v>0.9993</v>
@@ -13195,7 +13192,7 @@
         <v>0.9993</v>
       </c>
       <c r="G491">
-        <v>0.6073132316800103</v>
+        <v>0.6842806468068952</v>
       </c>
       <c r="H491">
         <v>0.9993</v>
@@ -15731,19 +15728,19 @@
         <v>15</v>
       </c>
       <c r="C589">
-        <v>33.11890811474259</v>
+        <v>40.85694740267934</v>
       </c>
       <c r="D589">
-        <v>18.01894893197226</v>
+        <v>18.86036647046424</v>
       </c>
       <c r="E589">
-        <v>0.9987</v>
+        <v>0.992</v>
       </c>
       <c r="F589">
-        <v>0.9987</v>
+        <v>0.992</v>
       </c>
       <c r="G589">
-        <v>0.7908413149493037</v>
+        <v>0.904963665701102</v>
       </c>
       <c r="H589">
         <v>0.9987</v>
@@ -18305,10 +18302,10 @@
         <v>16</v>
       </c>
       <c r="C688">
-        <v>28.01843343721627</v>
+        <v>28.00942554158634</v>
       </c>
       <c r="D688">
-        <v>16.56422974318342</v>
+        <v>16.55932295861207</v>
       </c>
       <c r="E688">
         <v>1.00016299</v>
@@ -18317,7 +18314,7 @@
         <v>1.00016299</v>
       </c>
       <c r="G688">
-        <v>0.2708953814312518</v>
+        <v>0.2892935311119793</v>
       </c>
       <c r="H688">
         <v>0.9993897</v>
@@ -20888,7 +20885,7 @@
         <v>1</v>
       </c>
       <c r="G787">
-        <v>0.05710018124847771</v>
+        <v>0.04331853251212658</v>
       </c>
       <c r="H787">
         <v>1</v>
@@ -23450,19 +23447,19 @@
         <v>18</v>
       </c>
       <c r="C886">
-        <v>35.75278262761136</v>
+        <v>35.75691573329998</v>
       </c>
       <c r="D886">
-        <v>19.45761115315375</v>
+        <v>19.45621659209236</v>
       </c>
       <c r="E886">
-        <v>0.99727644</v>
+        <v>0.99570457</v>
       </c>
       <c r="F886">
-        <v>0.99727644</v>
+        <v>0.99570457</v>
       </c>
       <c r="G886">
-        <v>0.3529568954465609</v>
+        <v>0.3681875296700767</v>
       </c>
       <c r="H886">
         <v>0.99927994</v>

</xml_diff>